<commit_message>
8.27 — Warehouse Operator Sidebar Redesign & Server Lockdown
</commit_message>
<xml_diff>
--- a/output/WMS_Импорт_РС УрФО Империал_2026-08-31.xlsx
+++ b/output/WMS_Импорт_РС УрФО Империал_2026-08-31.xlsx
@@ -624,14 +624,10 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Спальня Аврора Кровать 140 со встроенным основанием под матрас Дуб сонома/Белый упаковка 1/2</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>4603734803365</t>
-        </is>
-      </c>
+          <t>Аврора Кровать 140 с основанием 1/2 дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n"/>
       <c r="D4" s="2" t="n">
         <v>2</v>
       </c>
@@ -647,14 +643,10 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Спальня Аврора Кровать 140 со встроенным основанием под матрас Дуб сонома/Белый упаковка 2/2</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>4603734803372</t>
-        </is>
-      </c>
+          <t>Аврора Кровать 140 с основанием 2/2 дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
       <c r="D5" s="2" t="n">
         <v>2</v>
       </c>
@@ -5446,14 +5438,10 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>Прихожая Интер Зеркало 4мм 858х294 (полировка) упаковка Ун1/1</t>
-        </is>
-      </c>
-      <c r="C214" s="4" t="inlineStr">
-        <is>
-          <t>4673735517387</t>
-        </is>
-      </c>
+          <t>Зеркало 4мм 858х294 Прихожие дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="n"/>
       <c r="D214" s="2" t="n">
         <v>1</v>
       </c>
@@ -5889,14 +5877,10 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>Система Лацио Стекло 4мм 1310х376 (полировка) упаковка Ун1/1</t>
-        </is>
-      </c>
-      <c r="C235" s="4" t="inlineStr">
-        <is>
-          <t>4603745077526</t>
-        </is>
-      </c>
+          <t>ПФ Стекло 4 мм 1310х376 Лацио (полировка)</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="n"/>
       <c r="D235" s="2" t="n">
         <v>4</v>
       </c>
@@ -6190,14 +6174,10 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>Система Феникс Комплект крючков (3 шт) (фурнитура) Чёрный упаковка 1/1</t>
-        </is>
-      </c>
-      <c r="C250" s="4" t="inlineStr">
-        <is>
-          <t>4673770727673</t>
-        </is>
-      </c>
+          <t>Система Феникс Комплект крючков (3 шт) 1/1 черный</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="n"/>
       <c r="D250" s="2" t="n">
         <v>2</v>
       </c>
@@ -9310,7 +9290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9389,7 +9369,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9">
@@ -9409,7 +9389,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -9477,595 +9457,685 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Аврора Кровать 140 с основанием 1/2 дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Отсутствует в каталоге фабрики</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Аврора Кровать 140 с основанием 2/2 дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Отсутствует в каталоге фабрики</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>213</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Зеркало 4мм 858х294 Прихожие дуб сонома/белый</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Отсутствует в каталоге фабрики</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n">
+        <v>234</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>ПФ Стекло 4 мм 1310х376 Лацио (полировка)</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Отсутствует в каталоге фабрики</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>249</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Система Феникс Комплект крючков (3 шт) 1/1 черный</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Отсутствует в каталоге фабрики</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Позиции ниже не имеют заводского штрихкода в каталоге 1С 8. Если штрихкод не был внесен через веб-интерфейс перед выгрузкой, внесите его вручную в WMS или отсканируйте при фактической приемке на склад.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Таблица 2. Позиции без ШК (фурнитура / погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>Способ</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="14" t="n">
+    <row r="26">
+      <c r="A26" s="14" t="n">
         <v>206</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>04.002.20.312 Светильник LED накл. квадрат 12В серебристый серебристый</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C26" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="15" t="n">
+    <row r="27">
+      <c r="A27" s="15" t="n">
         <v>208</v>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Система Тринити Светильник мебельный Комод 1д/Пенал 1д/Шкаф 1д (3 Вт) упаковка Ун1/1</t>
         </is>
       </c>
-      <c r="C22" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="C27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="14" t="n">
+    <row r="28">
+      <c r="A28" s="14" t="n">
         <v>215</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Корзина Карго (K4PTJ023C 200 мм) с доводчиком упаковка Ун1/1 без цвета</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="C28" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="n">
+    <row r="29">
+      <c r="A29" s="15" t="n">
         <v>216</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>Корнер заглушка ЛВ 1/1 (476) белый</t>
         </is>
       </c>
-      <c r="C24" s="15" t="n">
+      <c r="C29" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="14" t="n">
+    <row r="30">
+      <c r="A30" s="14" t="n">
         <v>217</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Корнер заглушка ЛВ 1/1 алюминий</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="15" t="n">
+    <row r="31">
+      <c r="A31" s="15" t="n">
         <v>218</v>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>Корнер заглушка ЛВ 1/1 тростник</t>
         </is>
       </c>
-      <c r="C26" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="C31" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="14" t="n">
+    <row r="32">
+      <c r="A32" s="14" t="n">
         <v>219</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Корнер заглушка ПР 1/1 (476) белый</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C32" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="n">
+    <row r="33">
+      <c r="A33" s="15" t="n">
         <v>220</v>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>Корнер заглушка ПР 1/1 алюминий</t>
         </is>
       </c>
-      <c r="C28" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="C33" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="14" t="n">
+    <row r="34">
+      <c r="A34" s="14" t="n">
         <v>221</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Корнер заглушка ПР 1/1 тростник</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C34" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="15" t="n">
+    <row r="35">
+      <c r="A35" s="15" t="n">
         <v>222</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>Корнер угол внутр. 1/1 (476) белый</t>
         </is>
       </c>
-      <c r="C30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="C35" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="14" t="n">
+    <row r="36">
+      <c r="A36" s="14" t="n">
         <v>223</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Корнер угол внутр. 1/1 тростник</t>
         </is>
       </c>
-      <c r="C31" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="15" t="n">
+    <row r="37">
+      <c r="A37" s="15" t="n">
         <v>232</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Опора пласт. 150мм разборная ПГР черный</t>
         </is>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C37" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="14" t="n">
+    <row r="38">
+      <c r="A38" s="14" t="n">
         <v>236</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Планка 1516 угловая 38мм 1/1</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C38" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="15" t="n">
+    <row r="39">
+      <c r="A39" s="15" t="n">
         <v>237</v>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>Планка 1517 соединительная 38мм 1/1</t>
         </is>
       </c>
-      <c r="C34" s="15" t="n">
+      <c r="C39" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D39" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="n">
+    <row r="40">
+      <c r="A40" s="14" t="n">
         <v>238</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Планка 1519 торцевая 38мм 1/1</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
+      <c r="C40" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="15" t="n">
+    <row r="41">
+      <c r="A41" s="15" t="n">
         <v>239</v>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>Планка 1519(ч) торцевая 38мм 1/1</t>
         </is>
       </c>
-      <c r="C36" s="15" t="n">
+      <c r="C41" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="14" t="n">
+    <row r="42">
+      <c r="A42" s="14" t="n">
         <v>240</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Плинтус д/столешн. RUS 3 м 1/1 Дуб вотан (RUS-17)</t>
         </is>
       </c>
-      <c r="C37" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="C42" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="15" t="n">
+    <row r="43">
+      <c r="A43" s="15" t="n">
         <v>241</v>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>Плинтус д/столешн. RUS 3 м 1/1 Мрамор белый (RUS-15)</t>
         </is>
       </c>
-      <c r="C38" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+      <c r="C43" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="14" t="n">
+    <row r="44">
+      <c r="A44" s="14" t="n">
         <v>242</v>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Профиль соединительный 4мм 1/1</t>
         </is>
       </c>
-      <c r="C39" s="14" t="n">
+      <c r="C44" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="15" t="n">
+    <row r="45">
+      <c r="A45" s="15" t="n">
         <v>243</v>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B45" s="16" t="inlineStr">
         <is>
           <t>Профиль торцевой 4мм 1/1</t>
         </is>
       </c>
-      <c r="C40" s="15" t="n">
+      <c r="C45" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="14" t="n">
+    <row r="46">
+      <c r="A46" s="14" t="n">
         <v>244</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Профиль угловой 4мм 1/1</t>
         </is>
       </c>
-      <c r="C41" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C46" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="15" t="n">
+    <row r="47">
+      <c r="A47" s="15" t="n">
         <v>245</v>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Кухня Равенна Роял Цоколь пластиковый 100 мм Грей 3,2 м  упаковка Ун1/1</t>
         </is>
       </c>
-      <c r="C42" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="C47" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="14" t="n">
+    <row r="48">
+      <c r="A48" s="14" t="n">
         <v>246</v>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Кухня Равенна Роял Цоколь пластиковый 150 мм Скай 3,2 м  упаковка Ун1/1</t>
         </is>
       </c>
-      <c r="C43" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="C48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="15" t="n">
+    <row r="49">
+      <c r="A49" s="15" t="n">
         <v>286</v>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>Торцевая заглушка к цоколю 100 мм грей</t>
         </is>
       </c>
-      <c r="C44" s="15" t="n">
+      <c r="C49" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="14" t="n">
+    <row r="50">
+      <c r="A50" s="14" t="n">
         <v>287</v>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Угол 135 гр для цоколя 100 мм грей</t>
         </is>
       </c>
-      <c r="C45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="C50" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="15" t="n">
+    <row r="51">
+      <c r="A51" s="15" t="n">
         <v>288</v>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B51" s="16" t="inlineStr">
         <is>
           <t>Угол 90 гр для цоколя 100 мм грей</t>
         </is>
       </c>
-      <c r="C46" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="C51" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="14" t="n">
+    <row r="52">
+      <c r="A52" s="14" t="n">
         <v>289</v>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Угол 90 гр для цоколя 150 мм скай</t>
         </is>
       </c>
-      <c r="C47" s="14" t="n">
+      <c r="C52" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="15" t="n">
+    <row r="53">
+      <c r="A53" s="15" t="n">
         <v>314</v>
       </c>
-      <c r="B48" s="16" t="inlineStr">
+      <c r="B53" s="16" t="inlineStr">
         <is>
           <t>Фасады к кухне Равенна Роял Н20 Карго Грей упаковка 2/3 без цвета</t>
         </is>
       </c>
-      <c r="C48" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="C53" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="14" t="n">
+    <row r="54">
+      <c r="A54" s="14" t="n">
         <v>340</v>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Фурнитура Полка стеклянная 30/40/50/60/80 (полкодержатели 8 шт) без цвета</t>
         </is>
       </c>
-      <c r="C49" s="14" t="n">
+      <c r="C54" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="15" t="n">
+    <row r="55">
+      <c r="A55" s="15" t="n">
         <v>361</v>
       </c>
-      <c r="B50" s="16" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>Фурнитура к кухне Равенна Роял Н20 карго упаковка 3/3 без цвета</t>
         </is>
       </c>
-      <c r="C50" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="C55" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="14" t="n">
+    <row r="56">
+      <c r="A56" s="14" t="n">
         <v>384</v>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Ящик с доводчиком Н86 400 Белый упаковка Ун1/1</t>
         </is>
       </c>
-      <c r="C51" s="14" t="n">
+      <c r="C56" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Заводской ШК отсутствует (фурнитура/погонаж)</t>
         </is>
@@ -10073,10 +10143,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>